<commit_message>
6 second delay before signal is sent
</commit_message>
<xml_diff>
--- a/pricing calculator.xlsx
+++ b/pricing calculator.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>component</t>
   </si>
@@ -58,6 +58,33 @@
   </si>
   <si>
     <t>header</t>
+  </si>
+  <si>
+    <t>pcb</t>
+  </si>
+  <si>
+    <t>case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pcb screw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lid screw</t>
+  </si>
+  <si>
+    <t>o-ring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cost of components</t>
+  </si>
+  <si>
+    <t>shipping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fun profits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">price to charge</t>
   </si>
 </sst>
 </file>
@@ -92,7 +119,8 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -594,6 +622,10 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="14.00390625"/>
+    <col customWidth="1" min="8" max="8" width="20.00390625"/>
+    <col customWidth="1" min="10" max="10" width="11.57421875"/>
+    <col customWidth="1" min="11" max="11" width="13.421875"/>
+    <col customWidth="1" min="12" max="12" width="12.28125"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -621,7 +653,7 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <f>B2*C2</f>
+        <f t="shared" ref="D2:D9" si="0">B2*C2</f>
         <v>0.25600000000000001</v>
       </c>
     </row>
@@ -636,7 +668,7 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <f>B3*C3</f>
+        <f t="shared" si="0"/>
         <v>0.183</v>
       </c>
     </row>
@@ -651,7 +683,7 @@
         <v>1</v>
       </c>
       <c r="D4">
-        <f>B4*C4</f>
+        <f t="shared" si="0"/>
         <v>0.114</v>
       </c>
     </row>
@@ -666,7 +698,7 @@
         <v>1</v>
       </c>
       <c r="D5">
-        <f>B5*C5</f>
+        <f t="shared" si="0"/>
         <v>0.70099999999999996</v>
       </c>
     </row>
@@ -681,7 +713,7 @@
         <v>1</v>
       </c>
       <c r="D6">
-        <f>B6*C6</f>
+        <f t="shared" si="0"/>
         <v>0.54900000000000004</v>
       </c>
     </row>
@@ -696,7 +728,7 @@
         <v>1</v>
       </c>
       <c r="D7">
-        <f>B7*C7</f>
+        <f t="shared" si="0"/>
         <v>0.081000000000000003</v>
       </c>
     </row>
@@ -711,7 +743,7 @@
         <v>3</v>
       </c>
       <c r="D8">
-        <f>B8*C8</f>
+        <f t="shared" si="0"/>
         <v>0.096000000000000002</v>
       </c>
     </row>
@@ -726,7 +758,7 @@
         <v>1</v>
       </c>
       <c r="D9">
-        <f>B9*C9</f>
+        <f t="shared" si="0"/>
         <v>1.49</v>
       </c>
     </row>
@@ -741,7 +773,7 @@
         <v>1</v>
       </c>
       <c r="D10">
-        <f>B10*C10</f>
+        <f t="shared" ref="D10:D14" si="1">B10*C10</f>
         <v>5.9000000000000004</v>
       </c>
     </row>
@@ -756,27 +788,788 @@
         <v>2</v>
       </c>
       <c r="D11">
-        <f>B11*C11</f>
+        <f t="shared" si="1"/>
         <v>0.95999999999999996</v>
       </c>
     </row>
     <row r="12" ht="14.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>34.600000000000001</v>
+      </c>
+      <c r="C12">
+        <v>0.33333333333333331</v>
+      </c>
       <c r="D12">
-        <f>B12*C12</f>
+        <f t="shared" si="1"/>
+        <v>11.533333333333333</v>
+      </c>
+      <c r="E12"/>
+      <c r="F12"/>
+      <c r="G12"/>
+      <c r="H12"/>
+      <c r="I12"/>
+      <c r="J12"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12"/>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12"/>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" ht="14.25">
+      <c r="C13">
+        <v>1</v>
+      </c>
       <c r="D13">
-        <f>B13*C13</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
+      <c r="E13"/>
+      <c r="F13"/>
+      <c r="G13"/>
+      <c r="H13"/>
+      <c r="I13"/>
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13"/>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13"/>
     </row>
     <row r="14" ht="14.25">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="1">
+        <f>8.91/25</f>
+        <v>0.35639999999999999</v>
+      </c>
+      <c r="C14">
+        <v>4</v>
+      </c>
       <c r="D14">
-        <f>B14*C14</f>
+        <f t="shared" si="1"/>
+        <v>1.4256</v>
+      </c>
+      <c r="E14"/>
+      <c r="F14"/>
+      <c r="G14"/>
+      <c r="H14"/>
+      <c r="I14"/>
+      <c r="J14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+      <c r="N14"/>
+      <c r="O14"/>
+      <c r="P14"/>
+      <c r="Q14"/>
+      <c r="R14"/>
+      <c r="S14"/>
+      <c r="T14"/>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="A15" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15">
+        <f>13.32/50</f>
+        <v>0.26640000000000003</v>
+      </c>
+      <c r="C15">
+        <v>8</v>
+      </c>
+      <c r="D15">
+        <f>B15*C15</f>
+        <v>2.1312000000000002</v>
+      </c>
+      <c r="E15"/>
+      <c r="F15"/>
+      <c r="G15"/>
+      <c r="H15"/>
+      <c r="I15"/>
+      <c r="J15"/>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+      <c r="N15"/>
+      <c r="O15"/>
+      <c r="P15"/>
+      <c r="Q15"/>
+      <c r="R15"/>
+      <c r="S15"/>
+      <c r="T15"/>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="A16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="1">
+        <f>7.46/10</f>
+        <v>0.746</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16">
+        <f>B16*C16</f>
+        <v>0.746</v>
+      </c>
+      <c r="E16"/>
+      <c r="F16"/>
+      <c r="G16"/>
+      <c r="H16"/>
+      <c r="I16"/>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16"/>
+      <c r="O16"/>
+      <c r="P16"/>
+      <c r="Q16"/>
+      <c r="R16"/>
+      <c r="S16"/>
+      <c r="T16"/>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="A17"/>
+      <c r="B17"/>
+      <c r="C17"/>
+      <c r="D17">
+        <f>B17*C17</f>
         <v>0</v>
       </c>
+      <c r="E17"/>
+      <c r="F17"/>
+      <c r="G17"/>
+      <c r="H17"/>
+      <c r="I17"/>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17"/>
+      <c r="O17"/>
+      <c r="P17"/>
+      <c r="Q17"/>
+      <c r="R17"/>
+      <c r="S17"/>
+      <c r="T17"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="A18"/>
+      <c r="B18"/>
+      <c r="C18"/>
+      <c r="D18">
+        <f>B18*C18</f>
+        <v>0</v>
+      </c>
+      <c r="E18"/>
+      <c r="F18"/>
+      <c r="G18"/>
+      <c r="H18"/>
+      <c r="I18"/>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18"/>
+      <c r="O18"/>
+      <c r="P18"/>
+      <c r="Q18"/>
+      <c r="R18"/>
+      <c r="S18"/>
+      <c r="T18"/>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="E19"/>
+      <c r="F19"/>
+      <c r="G19"/>
+      <c r="H19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19"/>
+      <c r="O19"/>
+      <c r="P19"/>
+      <c r="Q19"/>
+      <c r="R19"/>
+      <c r="S19"/>
+      <c r="T19"/>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="E20"/>
+      <c r="F20"/>
+      <c r="G20"/>
+      <c r="H20">
+        <f>SUM(D2:D18)</f>
+        <v>26.166133333333335</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20"/>
+      <c r="O20"/>
+      <c r="P20"/>
+      <c r="Q20"/>
+      <c r="R20"/>
+      <c r="S20"/>
+      <c r="T20"/>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="E21"/>
+      <c r="F21"/>
+      <c r="G21"/>
+      <c r="H21"/>
+      <c r="I21"/>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21"/>
+      <c r="O21"/>
+      <c r="P21"/>
+      <c r="Q21"/>
+      <c r="R21"/>
+      <c r="S21"/>
+      <c r="T21"/>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="E22"/>
+      <c r="F22"/>
+      <c r="G22"/>
+      <c r="H22"/>
+      <c r="I22"/>
+      <c r="J22"/>
+      <c r="K22"/>
+      <c r="L22"/>
+      <c r="M22"/>
+      <c r="N22"/>
+      <c r="O22"/>
+      <c r="P22"/>
+      <c r="Q22"/>
+      <c r="R22"/>
+      <c r="S22"/>
+      <c r="T22"/>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="E23"/>
+      <c r="F23"/>
+      <c r="G23"/>
+      <c r="H23"/>
+      <c r="I23"/>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23"/>
+      <c r="O23"/>
+      <c r="P23"/>
+      <c r="Q23"/>
+      <c r="R23"/>
+      <c r="S23"/>
+      <c r="T23"/>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="E24"/>
+      <c r="F24"/>
+      <c r="G24"/>
+      <c r="H24"/>
+      <c r="I24"/>
+      <c r="J24"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24"/>
+      <c r="O24"/>
+      <c r="P24"/>
+      <c r="Q24"/>
+      <c r="R24"/>
+      <c r="S24"/>
+      <c r="T24"/>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="E25"/>
+      <c r="F25"/>
+      <c r="G25"/>
+      <c r="H25"/>
+      <c r="I25"/>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+      <c r="N25"/>
+      <c r="O25"/>
+      <c r="P25"/>
+      <c r="Q25"/>
+      <c r="R25"/>
+      <c r="S25"/>
+      <c r="T25"/>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="E26"/>
+      <c r="F26"/>
+      <c r="G26"/>
+      <c r="H26"/>
+      <c r="I26"/>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26"/>
+      <c r="O26"/>
+      <c r="P26"/>
+      <c r="Q26"/>
+      <c r="R26"/>
+      <c r="S26"/>
+      <c r="T26"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="E27"/>
+      <c r="F27"/>
+      <c r="G27"/>
+      <c r="H27"/>
+      <c r="I27"/>
+      <c r="J27"/>
+      <c r="K27"/>
+      <c r="L27"/>
+      <c r="M27"/>
+      <c r="N27"/>
+      <c r="O27"/>
+      <c r="P27"/>
+      <c r="Q27"/>
+      <c r="R27"/>
+      <c r="S27"/>
+      <c r="T27"/>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="E28"/>
+      <c r="F28"/>
+      <c r="G28"/>
+      <c r="H28"/>
+      <c r="I28"/>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28"/>
+      <c r="O28"/>
+      <c r="P28"/>
+      <c r="Q28"/>
+      <c r="R28"/>
+      <c r="S28"/>
+      <c r="T28"/>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="E29"/>
+      <c r="F29"/>
+      <c r="G29"/>
+      <c r="H29"/>
+      <c r="I29"/>
+      <c r="J29"/>
+      <c r="K29"/>
+      <c r="L29"/>
+      <c r="M29"/>
+      <c r="N29"/>
+      <c r="O29"/>
+      <c r="P29"/>
+      <c r="Q29"/>
+      <c r="R29"/>
+      <c r="S29"/>
+      <c r="T29"/>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="E30"/>
+      <c r="F30"/>
+      <c r="G30"/>
+      <c r="H30"/>
+      <c r="I30"/>
+      <c r="J30"/>
+      <c r="K30"/>
+      <c r="L30"/>
+      <c r="M30"/>
+      <c r="N30"/>
+      <c r="O30"/>
+      <c r="P30"/>
+      <c r="Q30"/>
+      <c r="R30"/>
+      <c r="S30"/>
+      <c r="T30"/>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="E31"/>
+      <c r="F31"/>
+      <c r="G31"/>
+      <c r="H31"/>
+      <c r="I31"/>
+      <c r="J31"/>
+      <c r="K31"/>
+      <c r="L31"/>
+      <c r="M31"/>
+      <c r="N31"/>
+      <c r="O31"/>
+      <c r="P31"/>
+      <c r="Q31"/>
+      <c r="R31"/>
+      <c r="S31"/>
+      <c r="T31"/>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="E32"/>
+      <c r="F32"/>
+      <c r="G32"/>
+      <c r="H32"/>
+      <c r="I32"/>
+      <c r="J32"/>
+      <c r="K32"/>
+      <c r="L32"/>
+      <c r="M32"/>
+      <c r="N32"/>
+      <c r="O32"/>
+      <c r="P32"/>
+      <c r="Q32"/>
+      <c r="R32"/>
+      <c r="S32"/>
+      <c r="T32"/>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="E33"/>
+      <c r="F33"/>
+      <c r="G33"/>
+      <c r="H33"/>
+      <c r="I33"/>
+      <c r="J33"/>
+      <c r="K33"/>
+      <c r="L33"/>
+      <c r="M33"/>
+      <c r="N33"/>
+      <c r="O33"/>
+      <c r="P33"/>
+      <c r="Q33"/>
+      <c r="R33"/>
+      <c r="S33"/>
+      <c r="T33"/>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="E34"/>
+      <c r="F34"/>
+      <c r="G34"/>
+      <c r="H34"/>
+      <c r="I34"/>
+      <c r="J34"/>
+      <c r="K34"/>
+      <c r="L34"/>
+      <c r="M34"/>
+      <c r="N34"/>
+      <c r="O34"/>
+      <c r="P34"/>
+      <c r="Q34"/>
+      <c r="R34"/>
+      <c r="S34"/>
+      <c r="T34"/>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="E35"/>
+      <c r="F35"/>
+      <c r="G35"/>
+      <c r="H35"/>
+      <c r="I35"/>
+      <c r="J35"/>
+      <c r="K35"/>
+      <c r="L35"/>
+      <c r="M35"/>
+      <c r="N35"/>
+      <c r="O35"/>
+      <c r="P35"/>
+      <c r="Q35"/>
+      <c r="R35"/>
+      <c r="S35"/>
+      <c r="T35"/>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="E36"/>
+      <c r="F36"/>
+      <c r="G36"/>
+      <c r="H36"/>
+      <c r="I36"/>
+      <c r="J36"/>
+      <c r="K36"/>
+      <c r="L36"/>
+      <c r="M36"/>
+      <c r="N36"/>
+      <c r="O36"/>
+      <c r="P36"/>
+      <c r="Q36"/>
+      <c r="R36"/>
+      <c r="S36"/>
+      <c r="T36"/>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="E37"/>
+      <c r="F37"/>
+      <c r="G37"/>
+      <c r="H37"/>
+      <c r="I37"/>
+      <c r="J37"/>
+      <c r="K37"/>
+      <c r="L37"/>
+      <c r="M37"/>
+      <c r="N37"/>
+      <c r="O37"/>
+      <c r="P37"/>
+      <c r="Q37"/>
+      <c r="R37"/>
+      <c r="S37"/>
+      <c r="T37"/>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="E38"/>
+      <c r="F38"/>
+      <c r="G38"/>
+      <c r="H38"/>
+      <c r="I38"/>
+      <c r="J38"/>
+      <c r="K38"/>
+      <c r="L38"/>
+      <c r="M38"/>
+      <c r="N38"/>
+      <c r="O38"/>
+      <c r="P38"/>
+      <c r="Q38"/>
+      <c r="R38"/>
+      <c r="S38"/>
+      <c r="T38"/>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="E39"/>
+      <c r="F39"/>
+      <c r="G39"/>
+      <c r="H39"/>
+      <c r="I39"/>
+      <c r="J39"/>
+      <c r="K39"/>
+      <c r="L39"/>
+      <c r="M39"/>
+      <c r="N39"/>
+      <c r="O39"/>
+      <c r="P39"/>
+      <c r="Q39"/>
+      <c r="R39"/>
+      <c r="S39"/>
+      <c r="T39"/>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="E40"/>
+      <c r="F40"/>
+      <c r="G40"/>
+      <c r="H40"/>
+      <c r="I40"/>
+      <c r="J40"/>
+      <c r="K40"/>
+      <c r="L40"/>
+      <c r="M40"/>
+      <c r="N40"/>
+      <c r="O40"/>
+      <c r="P40"/>
+      <c r="Q40"/>
+      <c r="R40"/>
+      <c r="S40"/>
+      <c r="T40"/>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="E41"/>
+      <c r="F41"/>
+      <c r="G41"/>
+      <c r="H41"/>
+      <c r="I41"/>
+      <c r="J41"/>
+      <c r="K41"/>
+      <c r="L41"/>
+      <c r="M41"/>
+      <c r="N41"/>
+      <c r="O41"/>
+      <c r="P41"/>
+      <c r="Q41"/>
+      <c r="R41"/>
+      <c r="S41"/>
+      <c r="T41"/>
+    </row>
+    <row r="42" ht="14.25">
+      <c r="E42"/>
+      <c r="F42"/>
+      <c r="G42"/>
+      <c r="H42"/>
+      <c r="I42"/>
+      <c r="J42"/>
+      <c r="K42"/>
+      <c r="L42"/>
+      <c r="M42"/>
+      <c r="N42"/>
+      <c r="O42"/>
+      <c r="P42"/>
+      <c r="Q42"/>
+      <c r="R42"/>
+      <c r="S42"/>
+      <c r="T42"/>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="E43"/>
+      <c r="F43"/>
+      <c r="G43"/>
+      <c r="H43"/>
+      <c r="I43"/>
+      <c r="J43"/>
+      <c r="K43"/>
+      <c r="L43"/>
+      <c r="M43"/>
+      <c r="N43"/>
+      <c r="O43"/>
+      <c r="P43"/>
+      <c r="Q43"/>
+      <c r="R43"/>
+      <c r="S43"/>
+      <c r="T43"/>
+    </row>
+    <row r="44" ht="14.25">
+      <c r="E44"/>
+      <c r="F44"/>
+      <c r="G44"/>
+      <c r="H44"/>
+      <c r="I44"/>
+      <c r="J44"/>
+      <c r="K44"/>
+      <c r="L44"/>
+      <c r="M44"/>
+      <c r="N44"/>
+      <c r="O44"/>
+      <c r="P44"/>
+      <c r="Q44"/>
+      <c r="R44"/>
+      <c r="S44"/>
+      <c r="T44"/>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="E45"/>
+      <c r="F45"/>
+      <c r="G45"/>
+      <c r="H45"/>
+      <c r="I45"/>
+      <c r="J45"/>
+      <c r="K45"/>
+      <c r="L45"/>
+      <c r="M45"/>
+      <c r="N45"/>
+      <c r="O45"/>
+      <c r="P45"/>
+      <c r="Q45"/>
+      <c r="R45"/>
+      <c r="S45"/>
+      <c r="T45"/>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="E46"/>
+      <c r="F46"/>
+      <c r="G46"/>
+      <c r="H46"/>
+      <c r="I46"/>
+      <c r="J46"/>
+      <c r="K46"/>
+      <c r="L46"/>
+      <c r="M46"/>
+      <c r="N46"/>
+      <c r="O46"/>
+      <c r="P46"/>
+      <c r="Q46"/>
+      <c r="R46"/>
+      <c r="S46"/>
+      <c r="T46"/>
+    </row>
+    <row r="47" ht="14.25">
+      <c r="E47"/>
+      <c r="F47"/>
+      <c r="G47"/>
+      <c r="H47"/>
+      <c r="I47"/>
+      <c r="J47"/>
+      <c r="K47"/>
+      <c r="L47"/>
+      <c r="M47"/>
+      <c r="N47"/>
+      <c r="O47"/>
+      <c r="P47"/>
+      <c r="Q47"/>
+      <c r="R47"/>
+      <c r="S47"/>
+      <c r="T47"/>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="E48"/>
+      <c r="F48"/>
+      <c r="G48"/>
+      <c r="H48"/>
+      <c r="I48"/>
+      <c r="J48"/>
+      <c r="K48"/>
+      <c r="L48"/>
+      <c r="M48"/>
+      <c r="N48"/>
+      <c r="O48"/>
+      <c r="P48"/>
+      <c r="Q48"/>
+      <c r="R48"/>
+      <c r="S48"/>
+      <c r="T48"/>
+    </row>
+    <row r="49" ht="14.25">
+      <c r="E49"/>
+      <c r="F49"/>
+      <c r="G49"/>
+      <c r="H49"/>
+      <c r="I49"/>
+      <c r="J49"/>
+      <c r="K49"/>
+      <c r="L49"/>
+      <c r="M49"/>
+      <c r="N49"/>
+      <c r="O49"/>
+      <c r="P49"/>
+      <c r="Q49"/>
+      <c r="R49"/>
+      <c r="S49"/>
+      <c r="T49"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
added the ability to abort poweroff if the user sets fob pin to high for just a little bit, will test on boat tomorrow
</commit_message>
<xml_diff>
--- a/pricing calculator.xlsx
+++ b/pricing calculator.xlsx
@@ -827,6 +827,10 @@
         <f t="shared" si="0"/>
         <v>0.096000000000000002</v>
       </c>
+      <c r="I8">
+        <f>IFERROR(G8/H8,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" t="s">
@@ -842,6 +846,10 @@
         <f t="shared" si="0"/>
         <v>1.49</v>
       </c>
+      <c r="I9">
+        <f>IFERROR(G9/H9,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
@@ -857,6 +865,10 @@
         <f t="shared" ref="D10:D18" si="2">B10*C10</f>
         <v>5.9000000000000004</v>
       </c>
+      <c r="I10">
+        <f>IFERROR(G10/H10,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
@@ -872,6 +884,10 @@
         <f t="shared" si="2"/>
         <v>0.95999999999999996</v>
       </c>
+      <c r="I11">
+        <f>IFERROR(G11/H11,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" t="s">
@@ -888,6 +904,10 @@
         <f t="shared" si="2"/>
         <v>11.533333333333333</v>
       </c>
+      <c r="I12">
+        <f>IFERROR(G12/H12,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
@@ -974,6 +994,10 @@
       </c>
     </row>
     <row r="19" ht="14.25">
+      <c r="D19">
+        <f>B19*C19</f>
+        <v>0</v>
+      </c>
       <c r="H19" s="1" t="s">
         <v>25</v>
       </c>
@@ -988,6 +1012,10 @@
       </c>
     </row>
     <row r="20" ht="14.25">
+      <c r="D20">
+        <f>B20*C20</f>
+        <v>0</v>
+      </c>
       <c r="H20">
         <f>SUM(D2:D18)</f>
         <v>30.420133333333336</v>
@@ -1003,6 +1031,42 @@
       <c r="K20">
         <f>H20+I20+J20</f>
         <v>108.61040000000001</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="D21">
+        <f>B21*C21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="D22">
+        <f>B22*C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="D23">
+        <f>B23*C23</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="D24">
+        <f>B24*C24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="D25">
+        <f>B25*C25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="D26">
+        <f>B26*C26</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>